<commit_message>
feat: 활물질(--active) 입자 구분을 tables.xlsx 및 make_tables.py에 추가
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tables.xlsx
+++ b/tables.xlsx
@@ -1,122 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="기초통계량 및 처리 시간 (개별 입자)" sheetId="1" r:id="rId4"/>
-    <sheet name="기초통계량 및 처리 시간 (LOT)" sheetId="2" r:id="rId5"/>
-    <sheet name="등급화" sheetId="3" r:id="rId6"/>
+    <sheet name="기초통계량 및 처리 시간 (개별 입자)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="기초통계량 및 처리 시간 (LOT)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="등급화" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
-  <si>
-    <t>기초통계량 및 처리 시간</t>
-  </si>
-  <si>
-    <t>지표 구분</t>
-  </si>
-  <si>
-    <t>입자 구분</t>
-  </si>
-  <si>
-    <t>평균</t>
-  </si>
-  <si>
-    <t>중앙값</t>
-  </si>
-  <si>
-    <t>표준편차</t>
-  </si>
-  <si>
-    <t>입도 (µm)</t>
-  </si>
-  <si>
-    <t>대입경</t>
-  </si>
-  <si>
-    <t>소입경</t>
-  </si>
-  <si>
-    <t>타원도</t>
-  </si>
-  <si>
-    <t>구형도</t>
-  </si>
-  <si>
-    <t>미분/깨짐 비율 (%)</t>
-  </si>
-  <si>
-    <t>기초통계량 및 처리 시간 (LOT 평균)</t>
-  </si>
-  <si>
-    <t>입도 표준편차 (µm)</t>
-  </si>
-  <si>
-    <t>입도 RMSD (µm)</t>
-  </si>
-  <si>
-    <t>이미지 당 처리 시간 (초)</t>
-  </si>
-  <si>
-    <t>등급화</t>
-  </si>
-  <si>
-    <t>정량화 지표</t>
-  </si>
-  <si>
-    <t>등급</t>
-  </si>
-  <si>
-    <t>입도 표준편차</t>
-  </si>
-  <si>
-    <t>범위</t>
-  </si>
-  <si>
-    <t>타원도 표준편차</t>
-  </si>
-  <si>
-    <t>미분/깨짐</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
+      <name val="Helvetica Neue"/>
+      <color indexed="8"/>
       <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color indexed="8"/>
       <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
+      <color indexed="8"/>
       <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -140,7 +66,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -422,118 +348,208 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="13"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+  <cellXfs count="41">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="22" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="ff000000"/>
@@ -1581,683 +1597,1004 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="5" width="16.3516" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col width="16.3516" customWidth="1" style="29" min="1" max="5"/>
+    <col width="16.3516" customWidth="1" style="29" min="6" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" customHeight="1">
-      <c r="A1" t="s" s="2">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
-    </row>
-    <row r="2" ht="21.05" customHeight="1">
-      <c r="A2" t="s" s="5">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s" s="5">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s" s="5">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s" s="5">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" ht="20.55" customHeight="1">
-      <c r="A3" t="s" s="6">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s" s="7">
-        <v>7</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-    </row>
-    <row r="4" ht="20.35" customHeight="1">
-      <c r="A4" s="9"/>
-      <c r="B4" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-    </row>
-    <row r="5" ht="20.35" customHeight="1">
-      <c r="A5" t="s" s="12">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-    </row>
-    <row r="6" ht="20.35" customHeight="1">
-      <c r="A6" s="13"/>
-      <c r="B6" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-    </row>
-    <row r="7" ht="20.35" customHeight="1">
-      <c r="A7" t="s" s="14">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-    </row>
-    <row r="8" ht="20.35" customHeight="1">
-      <c r="A8" s="15"/>
-      <c r="B8" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-    </row>
-    <row r="9" ht="20.35" customHeight="1">
-      <c r="A9" t="s" s="14">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-    </row>
-    <row r="10" ht="20.35" customHeight="1">
-      <c r="A10" s="15"/>
-      <c r="B10" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-    </row>
-    <row r="11" ht="20.35" customHeight="1">
-      <c r="A11" s="14"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-    </row>
-    <row r="12" ht="20.35" customHeight="1">
-      <c r="A12" s="15"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="15"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="15"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-    </row>
-    <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-    </row>
-    <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="15"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-    </row>
-    <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-    </row>
-    <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-    </row>
-    <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="15"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-    </row>
-    <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="15"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-    </row>
-    <row r="23" ht="20.05" customHeight="1">
-      <c r="A23" s="15"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-    </row>
-    <row r="24" ht="20.05" customHeight="1">
-      <c r="A24" s="15"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-    </row>
-    <row r="25" ht="20.05" customHeight="1">
-      <c r="A25" s="15"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
+    <row r="1" ht="29" customHeight="1" s="33">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>기초통계량 및 처리 시간</t>
+        </is>
+      </c>
+      <c r="B1" s="35" t="n"/>
+      <c r="C1" s="35" t="n"/>
+      <c r="D1" s="35" t="n"/>
+      <c r="E1" s="36" t="n"/>
+    </row>
+    <row r="2" ht="21.05" customHeight="1" s="33">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>지표 구분</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>입자 구분</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>평균</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>중앙값</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>표준편차</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20.35" customHeight="1" s="33">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>입도 (µm)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+    </row>
+    <row r="4" ht="20.35" customHeight="1" s="33">
+      <c r="A4" s="37" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+    </row>
+    <row r="5" ht="20.35" customHeight="1" s="33">
+      <c r="A5" s="38" t="n"/>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+    </row>
+    <row r="6" ht="20.35" customHeight="1" s="33">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>타원도</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+    </row>
+    <row r="7" ht="20.35" customHeight="1" s="33">
+      <c r="A7" s="37" t="n"/>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="20.35" customHeight="1" s="33">
+      <c r="A8" s="39" t="n"/>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="20.35" customHeight="1" s="33">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>구형도</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="20.35" customHeight="1" s="33">
+      <c r="A10" s="37" t="n"/>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="20.35" customHeight="1" s="33">
+      <c r="A11" s="38" t="n"/>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="20.35" customHeight="1" s="33">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>미분/깨짐 비율 (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="20.05" customHeight="1" s="33">
+      <c r="A13" s="37" t="n"/>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="20.05" customHeight="1" s="33">
+      <c r="A14" s="38" t="n"/>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="20.05" customHeight="1" s="33">
+      <c r="A15" s="14" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="20.05" customHeight="1" s="33">
+      <c r="A16" s="38" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="20.05" customHeight="1" s="33">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="20.05" customHeight="1" s="33">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="20.05" customHeight="1" s="33">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="20.05" customHeight="1" s="33">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+    </row>
+    <row r="21" ht="20.05" customHeight="1" s="33">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="20.05" customHeight="1" s="33">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="20.05" customHeight="1" s="33">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+    </row>
+    <row r="24" ht="20.05" customHeight="1" s="33">
+      <c r="A24" s="15" t="n"/>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+    </row>
+    <row r="25" ht="20.05" customHeight="1" s="33">
+      <c r="A25" s="15" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="n"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A15:A16"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A9:A11"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait" scale="72" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12 &amp;K000000&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="5" width="16.3516" style="17" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="17" customWidth="1"/>
+    <col width="16.3516" customWidth="1" style="29" min="1" max="5"/>
+    <col width="16.3516" customWidth="1" style="29" min="6" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" customHeight="1">
-      <c r="A1" t="s" s="2">
-        <v>12</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
-    </row>
-    <row r="2" ht="21.05" customHeight="1">
-      <c r="A2" t="s" s="5">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s" s="5">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s" s="5">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s" s="5">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" ht="20.55" customHeight="1">
-      <c r="A3" t="s" s="6">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s" s="7">
-        <v>7</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-    </row>
-    <row r="4" ht="20.35" customHeight="1">
-      <c r="A4" s="15"/>
-      <c r="B4" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-    </row>
-    <row r="5" ht="20.35" customHeight="1">
-      <c r="A5" t="s" s="14">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-    </row>
-    <row r="6" ht="20.35" customHeight="1">
-      <c r="A6" s="18"/>
-      <c r="B6" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-    </row>
-    <row r="7" ht="20.35" customHeight="1">
-      <c r="A7" t="s" s="14">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-    </row>
-    <row r="8" ht="20.35" customHeight="1">
-      <c r="A8" s="18"/>
-      <c r="B8" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-    </row>
-    <row r="9" ht="20.35" customHeight="1">
-      <c r="A9" t="s" s="19">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-    </row>
-    <row r="10" ht="20.35" customHeight="1">
-      <c r="A10" s="13"/>
-      <c r="B10" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-    </row>
-    <row r="11" ht="20.35" customHeight="1">
-      <c r="A11" t="s" s="14">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-    </row>
-    <row r="12" ht="20.35" customHeight="1">
-      <c r="A12" s="15"/>
-      <c r="B12" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" t="s" s="14">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="15"/>
-      <c r="B14" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" t="s" s="14">
-        <v>15</v>
-      </c>
-      <c r="B15" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="15"/>
-      <c r="B16" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-    </row>
-    <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="20"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="22"/>
-    </row>
-    <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="23"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="25"/>
-    </row>
-    <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="23"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="25"/>
-    </row>
-    <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="23"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="25"/>
-    </row>
-    <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="23"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="25"/>
-    </row>
-    <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="23"/>
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="25"/>
-    </row>
-    <row r="23" ht="20.05" customHeight="1">
-      <c r="A23" s="23"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
-    </row>
-    <row r="24" ht="20.05" customHeight="1">
-      <c r="A24" s="23"/>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="25"/>
-    </row>
-    <row r="25" ht="20.05" customHeight="1">
-      <c r="A25" s="26"/>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="28"/>
+    <row r="1" ht="29" customHeight="1" s="33">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>기초통계량 및 처리 시간 (LOT 평균)</t>
+        </is>
+      </c>
+      <c r="B1" s="35" t="n"/>
+      <c r="C1" s="35" t="n"/>
+      <c r="D1" s="35" t="n"/>
+      <c r="E1" s="36" t="n"/>
+    </row>
+    <row r="2" ht="21.05" customHeight="1" s="33">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>지표 구분</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>입자 구분</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>평균</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>중앙값</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>표준편차</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20.35" customHeight="1" s="33">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>입도 (µm)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+    </row>
+    <row r="4" ht="20.35" customHeight="1" s="33">
+      <c r="A4" s="37" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+    </row>
+    <row r="5" ht="20.35" customHeight="1" s="33">
+      <c r="A5" s="38" t="n"/>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+    </row>
+    <row r="6" ht="20.35" customHeight="1" s="33">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>입도 표준편차 (µm)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+    </row>
+    <row r="7" ht="20.35" customHeight="1" s="33">
+      <c r="A7" s="37" t="n"/>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="20.35" customHeight="1" s="33">
+      <c r="A8" s="38" t="n"/>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="20.35" customHeight="1" s="33">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>입도 RMSD (µm)</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="20.35" customHeight="1" s="33">
+      <c r="A10" s="37" t="n"/>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="20.35" customHeight="1" s="33">
+      <c r="A11" s="38" t="n"/>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="20.35" customHeight="1" s="33">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>타원도</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="20.05" customHeight="1" s="33">
+      <c r="A13" s="37" t="n"/>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="20.05" customHeight="1" s="33">
+      <c r="A14" s="39" t="n"/>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="20.05" customHeight="1" s="33">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>구형도</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="20.05" customHeight="1" s="33">
+      <c r="A16" s="37" t="n"/>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="20.05" customHeight="1" s="33">
+      <c r="A17" s="38" t="n"/>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="20.05" customHeight="1" s="33">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>미분/깨짐 비율 (%)</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="20.05" customHeight="1" s="33">
+      <c r="A19" s="37" t="n"/>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="20.05" customHeight="1" s="33">
+      <c r="A20" s="38" t="n"/>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+    </row>
+    <row r="21" ht="20.05" customHeight="1" s="33">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>이미지 당 처리 시간 (초)</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="20.05" customHeight="1" s="33">
+      <c r="A22" s="37" t="n"/>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="20.05" customHeight="1" s="33">
+      <c r="A23" s="38" t="n"/>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+    </row>
+    <row r="24" ht="20.05" customHeight="1" s="33">
+      <c r="A24" s="20" t="n"/>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="22" t="n"/>
+    </row>
+    <row r="25" ht="20.05" customHeight="1" s="33">
+      <c r="A25" s="40" t="n"/>
+      <c r="B25" s="24" t="n"/>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="25" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="25" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="40" t="n"/>
+      <c r="B27" s="24" t="n"/>
+      <c r="C27" s="24" t="n"/>
+      <c r="D27" s="24" t="n"/>
+      <c r="E27" s="25" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="25" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="25" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="25" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="25" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="26" t="n"/>
+      <c r="B32" s="27" t="n"/>
+      <c r="C32" s="27" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A15:A17"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A18:A20"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait" scale="72" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12 &amp;K000000&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="6" width="16.3516" style="29" customWidth="1"/>
-    <col min="7" max="16384" width="16.3516" style="29" customWidth="1"/>
+    <col width="16.3516" customWidth="1" style="29" min="1" max="6"/>
+    <col width="16.3516" customWidth="1" style="29" min="7" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" customHeight="1">
-      <c r="A1" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
-    </row>
-    <row r="2" ht="21.05" customHeight="1">
-      <c r="A2" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s" s="5">
-        <v>18</v>
-      </c>
-      <c r="C2" s="30">
+    <row r="1" ht="29" customHeight="1" s="33">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>등급화</t>
+        </is>
+      </c>
+      <c r="B1" s="35" t="n"/>
+      <c r="C1" s="35" t="n"/>
+      <c r="D1" s="35" t="n"/>
+      <c r="E1" s="35" t="n"/>
+      <c r="F1" s="36" t="n"/>
+    </row>
+    <row r="2" ht="21.05" customHeight="1" s="33">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>정량화 지표</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="C2" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="30">
+      <c r="D2" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="30">
+      <c r="E2" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="30">
+      <c r="F2" s="30" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" t="s" s="6">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s" s="7">
-        <v>20</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-    </row>
-    <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" s="15"/>
-      <c r="B4" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-    </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="B5" t="s" s="31">
-        <v>8</v>
-      </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-    </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" t="s" s="12">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s" s="7">
-        <v>20</v>
-      </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-    </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="32"/>
-      <c r="B7" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-    </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="13"/>
-      <c r="B8" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-    </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" t="s" s="14">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s" s="10">
-        <v>20</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-    </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="15"/>
-      <c r="B10" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-    </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="15"/>
-      <c r="B11" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-    </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" t="s" s="14">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s" s="10">
-        <v>20</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="15"/>
-      <c r="B13" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="15"/>
-      <c r="B14" t="s" s="10">
-        <v>8</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
+    <row r="3" ht="20.25" customHeight="1" s="33">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>입도 표준편차</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>범위</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+    </row>
+    <row r="4" ht="20.05" customHeight="1" s="33">
+      <c r="A4" s="37" t="n"/>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+    </row>
+    <row r="5" ht="20.05" customHeight="1" s="33">
+      <c r="A5" s="37" t="n"/>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="11" t="n"/>
+    </row>
+    <row r="6" ht="20.05" customHeight="1" s="33">
+      <c r="A6" s="38" t="n"/>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+    </row>
+    <row r="7" ht="20.05" customHeight="1" s="33">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>타원도 표준편차</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>범위</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="20.05" customHeight="1" s="33">
+      <c r="A8" s="37" t="n"/>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="20.05" customHeight="1" s="33">
+      <c r="A9" s="37" t="n"/>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="20.05" customHeight="1" s="33">
+      <c r="A10" s="39" t="n"/>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="20.05" customHeight="1" s="33">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>구형도</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>범위</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="20.05" customHeight="1" s="33">
+      <c r="A12" s="37" t="n"/>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="20.05" customHeight="1" s="33">
+      <c r="A13" s="37" t="n"/>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="20.05" customHeight="1" s="33">
+      <c r="A14" s="38" t="n"/>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>미분/깨짐</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>범위</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="n"/>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>활물질</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="n"/>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>대입경</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="n"/>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>소입경</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A7:A10"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A15:A18"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12 &amp;K000000&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>